<commit_message>
add all time parse & fix new players stats
</commit_message>
<xml_diff>
--- a/cska_stats.xlsx
+++ b/cska_stats.xlsx
@@ -60,7 +60,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="10"/>
@@ -68,19 +68,28 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="5"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -428,24 +437,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col width="23.7109375" customWidth="1" style="9" min="1" max="1"/>
-    <col width="15.7109375" customWidth="1" style="9" min="2" max="2"/>
-    <col width="26.5703125" customWidth="1" style="9" min="3" max="3"/>
-    <col width="8.85546875" customWidth="1" style="9" min="4" max="19"/>
-    <col width="8.85546875" customWidth="1" style="9" min="20" max="16384"/>
+    <col width="23.7109375" customWidth="1" style="12" min="1" max="1"/>
+    <col width="15.7109375" customWidth="1" style="12" min="2" max="2"/>
+    <col width="26.5703125" customWidth="1" style="12" min="3" max="3"/>
+    <col width="8.85546875" customWidth="1" style="12" min="4" max="22"/>
+    <col width="8.85546875" customWidth="1" style="12" min="23" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>СТАТИСТИКА ИГРОКОВ ЦСКА</t>
         </is>
       </c>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n"/>
@@ -468,284 +477,373 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Собкало Валерия</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>142</v>
+      <c r="B4" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>172</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Баева Юлия</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>116</v>
-      </c>
-      <c r="C5" s="2" t="n">
+      <c r="B5" s="4" t="n">
+        <v>135</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Семина Варвара</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Никитина Вероника</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Мурзалиева Альбина</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Козаченко Юлия</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
         <v>215</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Семина Варвара</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Никитина Вероника</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
+      <c r="C9" s="4" t="n">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Шинкарук Ирина</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Томилина Валентина</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Чигиринова Наталья</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>206</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Сабирова Карина</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Крупенникова Юлия</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Санталова Антонина</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>189</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Гаряева Юлия</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>117</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="17" ht="27.6" customHeight="1" s="12">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Илларионова Анастасия</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Левчина Екатерина</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Мурзалиева Альбина</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Козаченко Юлия</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>195</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Шинкарук Ирина</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Томилина Валентина</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Чигиринова Наталья</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>189</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Сабирова Карина</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>155</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Крупенникова Юлия</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
+      <c r="C18" s="4" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Явон Ольга</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>99</v>
+      </c>
+      <c r="C19" s="4" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Васильева Софья</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Захаренко Ева</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Санталова Антонина</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>172</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>660</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Гаряева Юлия</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="17" ht="27.6" customHeight="1" s="9">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Илларионова Анастасия</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>201</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Левчина Екатерина</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Явон Ольга</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Васильева Софья</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Захаренко Ева</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="C21" s="2" t="n">
+      <c r="C21" s="4" t="n">
         <v>34</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n"/>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Гаврилова Анна</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n"/>
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Михайличенко Елена</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n">
+        <v>111</v>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>499</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Кузнецова Наталья</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Ихнева Алена</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" ht="28.5" customHeight="1" s="12">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Островская Александра</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Пукас Арина</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>Верещак Анна</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="B30" t="n">
+        <v>42</v>
+      </c>
+      <c r="C30" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>Аношкина Эвелина</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="B31" t="n">
+        <v>91</v>
+      </c>
+      <c r="C31" t="n">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>Маркина Полина</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
-        <v>215</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>1364</v>
+      <c r="B32" t="n">
+        <v>234</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Крутикова Карина</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>